<commit_message>
Checklist: aba Manager reflete a base ja construida no esqueleto
Depois de portar o nucleo de seguranca para manager/, 16 controles do Manager
sao Feito (com teste), 2 Em andamento (RBAC, CORS: base pronta, falta acabar),
o resto segue Planejado.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/specs/Checklist-Seguranca-por-Servico.xlsx
+++ b/specs/Checklist-Seguranca-por-Servico.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -74,6 +74,11 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="008A6100"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
     </font>
   </fonts>
   <fills count="10">
@@ -150,7 +155,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -195,13 +200,16 @@
     <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -778,10 +786,10 @@
         </is>
       </c>
       <c r="B24" s="15" t="n">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="C24" s="15" t="n">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="D24" s="15" t="n">
         <v>49</v>
@@ -846,7 +854,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>5 de 49 controles feitos. 44 em planejamento. Modelo pronto e testado: Print.</t>
+          <t>16 de 49 controles feitos. Modelo pronto e testado: Print. Base de seguranca ja construida e testada em manager/ (14 testes).</t>
         </is>
       </c>
     </row>
@@ -913,12 +921,12 @@
       </c>
       <c r="E5" s="16" t="inlineStr">
         <is>
-          <t>Nada, ja implementado.</t>
+          <t>Feito no esqueleto (manager/), com teste em teste-manager.js.</t>
         </is>
       </c>
       <c r="F5" s="14" t="inlineStr">
         <is>
-          <t>Feito no Print</t>
+          <t>Feito no Manager</t>
         </is>
       </c>
       <c r="G5" s="17" t="inlineStr">
@@ -953,12 +961,12 @@
       </c>
       <c r="E6" s="16" t="inlineStr">
         <is>
-          <t>Nada, ja implementado.</t>
+          <t>Feito no esqueleto (manager/), com teste em teste-manager.js.</t>
         </is>
       </c>
       <c r="F6" s="14" t="inlineStr">
         <is>
-          <t>Feito no Print</t>
+          <t>Feito no Manager</t>
         </is>
       </c>
       <c r="G6" s="17" t="inlineStr">
@@ -993,12 +1001,12 @@
       </c>
       <c r="E7" s="16" t="inlineStr">
         <is>
-          <t>Nada, ja implementado.</t>
+          <t>Feito no esqueleto (manager/), com teste em teste-manager.js.</t>
         </is>
       </c>
       <c r="F7" s="14" t="inlineStr">
         <is>
-          <t>Feito no Print</t>
+          <t>Feito no Manager</t>
         </is>
       </c>
       <c r="G7" s="17" t="inlineStr">
@@ -1033,12 +1041,12 @@
       </c>
       <c r="E8" s="16" t="inlineStr">
         <is>
-          <t>Nada, ja implementado.</t>
+          <t>Feito no esqueleto (manager/), com teste em teste-manager.js.</t>
         </is>
       </c>
       <c r="F8" s="14" t="inlineStr">
         <is>
-          <t>Feito no Print</t>
+          <t>Feito no Manager</t>
         </is>
       </c>
       <c r="G8" s="17" t="inlineStr">
@@ -1073,12 +1081,12 @@
       </c>
       <c r="E9" s="16" t="inlineStr">
         <is>
-          <t>Nada, ja implementado.</t>
+          <t>Feito no esqueleto (manager/), com teste em teste-manager.js.</t>
         </is>
       </c>
       <c r="F9" s="14" t="inlineStr">
         <is>
-          <t>Feito no Print</t>
+          <t>Feito no Manager</t>
         </is>
       </c>
       <c r="G9" s="17" t="inlineStr">
@@ -1113,22 +1121,22 @@
       </c>
       <c r="E10" s="16" t="inlineStr">
         <is>
-          <t>Plugar cifra.js na gravacao de conteudo do servico.</t>
-        </is>
-      </c>
-      <c r="F10" s="18" t="inlineStr">
-        <is>
-          <t>Copiar do Print</t>
-        </is>
-      </c>
-      <c r="G10" s="19" t="inlineStr">
-        <is>
-          <t>Planejado</t>
-        </is>
-      </c>
-      <c r="H10" s="15" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+          <t>Feito no esqueleto (manager/), com teste em teste-manager.js.</t>
+        </is>
+      </c>
+      <c r="F10" s="14" t="inlineStr">
+        <is>
+          <t>Feito no Manager</t>
+        </is>
+      </c>
+      <c r="G10" s="17" t="inlineStr">
+        <is>
+          <t>Feito</t>
+        </is>
+      </c>
+      <c r="H10" s="17" t="inlineStr">
+        <is>
+          <t>Feito</t>
         </is>
       </c>
     </row>
@@ -1156,7 +1164,7 @@
           <t>Dar prazo de validade ao objeto do servico.</t>
         </is>
       </c>
-      <c r="F11" s="20" t="inlineStr">
+      <c r="F11" s="18" t="inlineStr">
         <is>
           <t>Adaptar do Print</t>
         </is>
@@ -1196,7 +1204,7 @@
           <t>Reusar a poda por prazo no caminho de leitura.</t>
         </is>
       </c>
-      <c r="F12" s="18" t="inlineStr">
+      <c r="F12" s="20" t="inlineStr">
         <is>
           <t>Copiar do Print</t>
         </is>
@@ -1236,7 +1244,7 @@
           <t>Excluir tem que apagar metadado e objeto juntos.</t>
         </is>
       </c>
-      <c r="F13" s="20" t="inlineStr">
+      <c r="F13" s="18" t="inlineStr">
         <is>
           <t>Adaptar do Print</t>
         </is>
@@ -1273,22 +1281,22 @@
       </c>
       <c r="E14" s="16" t="inlineStr">
         <is>
-          <t>Segredos so em variavel de ambiente; nunca no repo.</t>
-        </is>
-      </c>
-      <c r="F14" s="18" t="inlineStr">
-        <is>
-          <t>Copiar do Print</t>
-        </is>
-      </c>
-      <c r="G14" s="19" t="inlineStr">
-        <is>
-          <t>Planejado</t>
-        </is>
-      </c>
-      <c r="H14" s="15" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+          <t>Feito no esqueleto (manager/), com teste em teste-manager.js.</t>
+        </is>
+      </c>
+      <c r="F14" s="14" t="inlineStr">
+        <is>
+          <t>Feito no Manager</t>
+        </is>
+      </c>
+      <c r="G14" s="17" t="inlineStr">
+        <is>
+          <t>Feito</t>
+        </is>
+      </c>
+      <c r="H14" s="17" t="inlineStr">
+        <is>
+          <t>Feito</t>
         </is>
       </c>
     </row>
@@ -1313,22 +1321,22 @@
       </c>
       <c r="E15" s="16" t="inlineStr">
         <is>
-          <t>Criar tabela de auditoria e registrar acoes criticas.</t>
-        </is>
-      </c>
-      <c r="F15" s="18" t="inlineStr">
-        <is>
-          <t>Copiar do Print</t>
-        </is>
-      </c>
-      <c r="G15" s="19" t="inlineStr">
-        <is>
-          <t>Planejado</t>
-        </is>
-      </c>
-      <c r="H15" s="15" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+          <t>Feito no esqueleto (manager/), com teste em teste-manager.js.</t>
+        </is>
+      </c>
+      <c r="F15" s="14" t="inlineStr">
+        <is>
+          <t>Feito no Manager</t>
+        </is>
+      </c>
+      <c r="G15" s="17" t="inlineStr">
+        <is>
+          <t>Feito</t>
+        </is>
+      </c>
+      <c r="H15" s="17" t="inlineStr">
+        <is>
+          <t>Feito</t>
         </is>
       </c>
     </row>
@@ -1353,22 +1361,22 @@
       </c>
       <c r="E16" s="16" t="inlineStr">
         <is>
-          <t>Reusar papeis: admin, gestor, consultor, leitor.</t>
-        </is>
-      </c>
-      <c r="F16" s="18" t="inlineStr">
-        <is>
-          <t>Copiar do Print</t>
-        </is>
-      </c>
-      <c r="G16" s="19" t="inlineStr">
-        <is>
-          <t>Planejado</t>
-        </is>
-      </c>
-      <c r="H16" s="15" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+          <t>Papel e sessao ja prontos (a sessao cai quando o vinculo some); falta barrar acao por papel, como no Print.</t>
+        </is>
+      </c>
+      <c r="F16" s="20" t="inlineStr">
+        <is>
+          <t>Base pronta, falta acabar</t>
+        </is>
+      </c>
+      <c r="G16" s="21" t="inlineStr">
+        <is>
+          <t>Em andamento</t>
+        </is>
+      </c>
+      <c r="H16" s="21" t="inlineStr">
+        <is>
+          <t>Em andamento</t>
         </is>
       </c>
     </row>
@@ -1393,22 +1401,22 @@
       </c>
       <c r="E17" s="16" t="inlineStr">
         <is>
-          <t>Registrar acesso, criacao, download e exclusao por cliente.</t>
-        </is>
-      </c>
-      <c r="F17" s="18" t="inlineStr">
-        <is>
-          <t>Copiar do Print</t>
-        </is>
-      </c>
-      <c r="G17" s="19" t="inlineStr">
-        <is>
-          <t>Planejado</t>
-        </is>
-      </c>
-      <c r="H17" s="15" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+          <t>Feito no esqueleto (manager/), com teste em teste-manager.js.</t>
+        </is>
+      </c>
+      <c r="F17" s="14" t="inlineStr">
+        <is>
+          <t>Feito no Manager</t>
+        </is>
+      </c>
+      <c r="G17" s="17" t="inlineStr">
+        <is>
+          <t>Feito</t>
+        </is>
+      </c>
+      <c r="H17" s="17" t="inlineStr">
+        <is>
+          <t>Feito</t>
         </is>
       </c>
     </row>
@@ -1433,22 +1441,22 @@
       </c>
       <c r="E18" s="16" t="inlineStr">
         <is>
-          <t>Reusar o freio (429) por conta e por origem.</t>
-        </is>
-      </c>
-      <c r="F18" s="18" t="inlineStr">
-        <is>
-          <t>Copiar do Print</t>
-        </is>
-      </c>
-      <c r="G18" s="19" t="inlineStr">
-        <is>
-          <t>Planejado</t>
-        </is>
-      </c>
-      <c r="H18" s="15" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+          <t>Feito no esqueleto (manager/), com teste em teste-manager.js.</t>
+        </is>
+      </c>
+      <c r="F18" s="14" t="inlineStr">
+        <is>
+          <t>Feito no Manager</t>
+        </is>
+      </c>
+      <c r="G18" s="17" t="inlineStr">
+        <is>
+          <t>Feito</t>
+        </is>
+      </c>
+      <c r="H18" s="17" t="inlineStr">
+        <is>
+          <t>Feito</t>
         </is>
       </c>
     </row>
@@ -1473,22 +1481,22 @@
       </c>
       <c r="E19" s="16" t="inlineStr">
         <is>
-          <t>Reusar a validacao e o parse de corpo do api.js.</t>
-        </is>
-      </c>
-      <c r="F19" s="18" t="inlineStr">
-        <is>
-          <t>Copiar do Print</t>
-        </is>
-      </c>
-      <c r="G19" s="19" t="inlineStr">
-        <is>
-          <t>Planejado</t>
-        </is>
-      </c>
-      <c r="H19" s="15" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+          <t>Feito no esqueleto (manager/), com teste em teste-manager.js.</t>
+        </is>
+      </c>
+      <c r="F19" s="14" t="inlineStr">
+        <is>
+          <t>Feito no Manager</t>
+        </is>
+      </c>
+      <c r="G19" s="17" t="inlineStr">
+        <is>
+          <t>Feito</t>
+        </is>
+      </c>
+      <c r="H19" s="17" t="inlineStr">
+        <is>
+          <t>Feito</t>
         </is>
       </c>
     </row>
@@ -1513,22 +1521,22 @@
       </c>
       <c r="E20" s="16" t="inlineStr">
         <is>
-          <t>Reusar o limite de tamanho de corpo e upload.</t>
-        </is>
-      </c>
-      <c r="F20" s="18" t="inlineStr">
-        <is>
-          <t>Copiar do Print</t>
-        </is>
-      </c>
-      <c r="G20" s="19" t="inlineStr">
-        <is>
-          <t>Planejado</t>
-        </is>
-      </c>
-      <c r="H20" s="15" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+          <t>Feito no esqueleto (manager/), com teste em teste-manager.js.</t>
+        </is>
+      </c>
+      <c r="F20" s="14" t="inlineStr">
+        <is>
+          <t>Feito no Manager</t>
+        </is>
+      </c>
+      <c r="G20" s="17" t="inlineStr">
+        <is>
+          <t>Feito</t>
+        </is>
+      </c>
+      <c r="H20" s="17" t="inlineStr">
+        <is>
+          <t>Feito</t>
         </is>
       </c>
     </row>
@@ -1556,7 +1564,7 @@
           <t>Aceitar so os tipos de arquivo da lista.</t>
         </is>
       </c>
-      <c r="F21" s="18" t="inlineStr">
+      <c r="F21" s="20" t="inlineStr">
         <is>
           <t>Copiar do Print</t>
         </is>
@@ -1593,22 +1601,22 @@
       </c>
       <c r="E22" s="16" t="inlineStr">
         <is>
-          <t>Fechar CORS para as origens conhecidas.</t>
-        </is>
-      </c>
-      <c r="F22" s="18" t="inlineStr">
-        <is>
-          <t>Copiar do Print</t>
-        </is>
-      </c>
-      <c r="G22" s="19" t="inlineStr">
-        <is>
-          <t>Planejado</t>
-        </is>
-      </c>
-      <c r="H22" s="15" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+          <t>Sem CORS aberto por padrao (cross-origin ja bloqueado); falta a regra explicita de origem e o teste dela.</t>
+        </is>
+      </c>
+      <c r="F22" s="20" t="inlineStr">
+        <is>
+          <t>Base pronta, falta acabar</t>
+        </is>
+      </c>
+      <c r="G22" s="21" t="inlineStr">
+        <is>
+          <t>Em andamento</t>
+        </is>
+      </c>
+      <c r="H22" s="21" t="inlineStr">
+        <is>
+          <t>Em andamento</t>
         </is>
       </c>
     </row>
@@ -1633,22 +1641,22 @@
       </c>
       <c r="E23" s="16" t="inlineStr">
         <is>
-          <t>Copiar os cabecalhos de seguranca do servidor.js.</t>
-        </is>
-      </c>
-      <c r="F23" s="18" t="inlineStr">
-        <is>
-          <t>Copiar do Print</t>
-        </is>
-      </c>
-      <c r="G23" s="19" t="inlineStr">
-        <is>
-          <t>Planejado</t>
-        </is>
-      </c>
-      <c r="H23" s="15" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+          <t>Feito no esqueleto (manager/), com teste em teste-manager.js.</t>
+        </is>
+      </c>
+      <c r="F23" s="14" t="inlineStr">
+        <is>
+          <t>Feito no Manager</t>
+        </is>
+      </c>
+      <c r="G23" s="17" t="inlineStr">
+        <is>
+          <t>Feito</t>
+        </is>
+      </c>
+      <c r="H23" s="17" t="inlineStr">
+        <is>
+          <t>Feito</t>
         </is>
       </c>
     </row>
@@ -1673,22 +1681,22 @@
       </c>
       <c r="E24" s="16" t="inlineStr">
         <is>
-          <t>Erro nunca devolve stack; 500 controlado.</t>
-        </is>
-      </c>
-      <c r="F24" s="18" t="inlineStr">
-        <is>
-          <t>Copiar do Print</t>
-        </is>
-      </c>
-      <c r="G24" s="19" t="inlineStr">
-        <is>
-          <t>Planejado</t>
-        </is>
-      </c>
-      <c r="H24" s="15" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+          <t>Feito no esqueleto (manager/), com teste em teste-manager.js.</t>
+        </is>
+      </c>
+      <c r="F24" s="14" t="inlineStr">
+        <is>
+          <t>Feito no Manager</t>
+        </is>
+      </c>
+      <c r="G24" s="17" t="inlineStr">
+        <is>
+          <t>Feito</t>
+        </is>
+      </c>
+      <c r="H24" s="17" t="inlineStr">
+        <is>
+          <t>Feito</t>
         </is>
       </c>
     </row>
@@ -1713,22 +1721,22 @@
       </c>
       <c r="E25" s="16" t="inlineStr">
         <is>
-          <t>Reusar o backup do admin.js.</t>
-        </is>
-      </c>
-      <c r="F25" s="18" t="inlineStr">
-        <is>
-          <t>Copiar do Print</t>
-        </is>
-      </c>
-      <c r="G25" s="19" t="inlineStr">
-        <is>
-          <t>Planejado</t>
-        </is>
-      </c>
-      <c r="H25" s="15" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+          <t>Feito no esqueleto (manager/), com teste em teste-manager.js.</t>
+        </is>
+      </c>
+      <c r="F25" s="14" t="inlineStr">
+        <is>
+          <t>Feito no Manager</t>
+        </is>
+      </c>
+      <c r="G25" s="17" t="inlineStr">
+        <is>
+          <t>Feito</t>
+        </is>
+      </c>
+      <c r="H25" s="17" t="inlineStr">
+        <is>
+          <t>Feito</t>
         </is>
       </c>
     </row>
@@ -1753,22 +1761,22 @@
       </c>
       <c r="E26" s="16" t="inlineStr">
         <is>
-          <t>Reusar teste-backup.js: destruir e restaurar de verdade.</t>
-        </is>
-      </c>
-      <c r="F26" s="18" t="inlineStr">
-        <is>
-          <t>Copiar do Print</t>
-        </is>
-      </c>
-      <c r="G26" s="19" t="inlineStr">
-        <is>
-          <t>Planejado</t>
-        </is>
-      </c>
-      <c r="H26" s="15" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+          <t>Feito no esqueleto (manager/), com teste em teste-manager.js.</t>
+        </is>
+      </c>
+      <c r="F26" s="14" t="inlineStr">
+        <is>
+          <t>Feito no Manager</t>
+        </is>
+      </c>
+      <c r="G26" s="17" t="inlineStr">
+        <is>
+          <t>Feito</t>
+        </is>
+      </c>
+      <c r="H26" s="17" t="inlineStr">
+        <is>
+          <t>Feito</t>
         </is>
       </c>
     </row>
@@ -1796,7 +1804,7 @@
           <t>Chaves e banco separados por ambiente (dev/homolog/prod).</t>
         </is>
       </c>
-      <c r="F27" s="21" t="inlineStr">
+      <c r="F27" s="22" t="inlineStr">
         <is>
           <t>Ligar no CI / infra</t>
         </is>
@@ -1836,7 +1844,7 @@
           <t>Rodar os mesmos testes no CI antes de subir.</t>
         </is>
       </c>
-      <c r="F28" s="21" t="inlineStr">
+      <c r="F28" s="22" t="inlineStr">
         <is>
           <t>Ligar no CI / infra</t>
         </is>
@@ -1876,7 +1884,7 @@
           <t>Exigir revisao de PR antes do main.</t>
         </is>
       </c>
-      <c r="F29" s="21" t="inlineStr">
+      <c r="F29" s="22" t="inlineStr">
         <is>
           <t>Ligar no CI / infra</t>
         </is>
@@ -1916,7 +1924,7 @@
           <t>Ligar o codeql.yml no repositorio do servico.</t>
         </is>
       </c>
-      <c r="F30" s="21" t="inlineStr">
+      <c r="F30" s="22" t="inlineStr">
         <is>
           <t>Ligar no CI / infra</t>
         </is>
@@ -1956,7 +1964,7 @@
           <t>Rodar npm audit (ou equivalente) no CI.</t>
         </is>
       </c>
-      <c r="F31" s="21" t="inlineStr">
+      <c r="F31" s="22" t="inlineStr">
         <is>
           <t>Ligar no CI / infra</t>
         </is>
@@ -1996,7 +2004,7 @@
           <t>Ligar o secret scanning do GitHub e revisar o .gitignore.</t>
         </is>
       </c>
-      <c r="F32" s="21" t="inlineStr">
+      <c r="F32" s="22" t="inlineStr">
         <is>
           <t>Ligar no CI / infra</t>
         </is>
@@ -2036,7 +2044,7 @@
           <t>Fixar versoes e ligar o Dependabot.</t>
         </is>
       </c>
-      <c r="F33" s="21" t="inlineStr">
+      <c r="F33" s="22" t="inlineStr">
         <is>
           <t>Ligar no CI / infra</t>
         </is>
@@ -2076,7 +2084,7 @@
           <t>Deixar a identidade pronta para SSO (sso.js ja prepara).</t>
         </is>
       </c>
-      <c r="F34" s="18" t="inlineStr">
+      <c r="F34" s="20" t="inlineStr">
         <is>
           <t>Copiar do Print</t>
         </is>
@@ -2116,7 +2124,7 @@
           <t>Escrever o processo de resposta a incidente (vale p/ os tres).</t>
         </is>
       </c>
-      <c r="F35" s="22" t="inlineStr">
+      <c r="F35" s="23" t="inlineStr">
         <is>
           <t>Documento (escrever 1x)</t>
         </is>
@@ -2156,7 +2164,7 @@
           <t>Formalizar o tratamento LGPD e reusar o mascaramento de dado sensivel.</t>
         </is>
       </c>
-      <c r="F36" s="22" t="inlineStr">
+      <c r="F36" s="23" t="inlineStr">
         <is>
           <t>Documento (escrever 1x)</t>
         </is>
@@ -2196,7 +2204,7 @@
           <t>Listar quais dados o servico trata (curto, por servico).</t>
         </is>
       </c>
-      <c r="F37" s="22" t="inlineStr">
+      <c r="F37" s="23" t="inlineStr">
         <is>
           <t>Documento (escrever 1x)</t>
         </is>
@@ -2236,7 +2244,7 @@
           <t>Listar terceiros que processam dados (Railway etc, vale p/ os tres).</t>
         </is>
       </c>
-      <c r="F38" s="22" t="inlineStr">
+      <c r="F38" s="23" t="inlineStr">
         <is>
           <t>Documento (escrever 1x)</t>
         </is>
@@ -2276,7 +2284,7 @@
           <t>Copiar sso.js e teste-sso.js e apontar para o provedor do cliente.</t>
         </is>
       </c>
-      <c r="F39" s="18" t="inlineStr">
+      <c r="F39" s="20" t="inlineStr">
         <is>
           <t>Copiar do Print</t>
         </is>
@@ -2316,7 +2324,7 @@
           <t>Adaptar o dast.js as rotas do servico e rodar no CI.</t>
         </is>
       </c>
-      <c r="F40" s="21" t="inlineStr">
+      <c r="F40" s="22" t="inlineStr">
         <is>
           <t>Ligar no CI / infra</t>
         </is>
@@ -2356,7 +2364,7 @@
           <t>Agendar pentest externo (fora do time).</t>
         </is>
       </c>
-      <c r="F41" s="23" t="inlineStr">
+      <c r="F41" s="24" t="inlineStr">
         <is>
           <t>Arquitetura / externo</t>
         </is>
@@ -2396,7 +2404,7 @@
           <t>Se o servico usa modelo, reusar injecao.js; senao, nao se aplica.</t>
         </is>
       </c>
-      <c r="F42" s="18" t="inlineStr">
+      <c r="F42" s="20" t="inlineStr">
         <is>
           <t>Copiar do Print</t>
         </is>
@@ -2436,7 +2444,7 @@
           <t>Reusar injecao.js: conteudo externo entra como dado, nunca ordem.</t>
         </is>
       </c>
-      <c r="F43" s="18" t="inlineStr">
+      <c r="F43" s="20" t="inlineStr">
         <is>
           <t>Copiar do Print</t>
         </is>
@@ -2476,7 +2484,7 @@
           <t>O modelo nao executa acao; so descreve.</t>
         </is>
       </c>
-      <c r="F44" s="23" t="inlineStr">
+      <c r="F44" s="24" t="inlineStr">
         <is>
           <t>Arquitetura / externo</t>
         </is>
@@ -2516,7 +2524,7 @@
           <t>Reusar a conferencia de saida do injecao.js.</t>
         </is>
       </c>
-      <c r="F45" s="18" t="inlineStr">
+      <c r="F45" s="20" t="inlineStr">
         <is>
           <t>Copiar do Print</t>
         </is>
@@ -2556,7 +2564,7 @@
           <t>Documentar a arquitetura e os controles do servico.</t>
         </is>
       </c>
-      <c r="F46" s="22" t="inlineStr">
+      <c r="F46" s="23" t="inlineStr">
         <is>
           <t>Documento (escrever 1x)</t>
         </is>
@@ -2596,7 +2604,7 @@
           <t>Desenhar o fluxo de dados do servico.</t>
         </is>
       </c>
-      <c r="F47" s="22" t="inlineStr">
+      <c r="F47" s="23" t="inlineStr">
         <is>
           <t>Documento (escrever 1x)</t>
         </is>
@@ -2636,7 +2644,7 @@
           <t>Marcar as fronteiras de confianca do servico.</t>
         </is>
       </c>
-      <c r="F48" s="22" t="inlineStr">
+      <c r="F48" s="23" t="inlineStr">
         <is>
           <t>Documento (escrever 1x)</t>
         </is>
@@ -2676,7 +2684,7 @@
           <t>FAQ de seguranca padrao (vale p/ os tres).</t>
         </is>
       </c>
-      <c r="F49" s="22" t="inlineStr">
+      <c r="F49" s="23" t="inlineStr">
         <is>
           <t>Documento (escrever 1x)</t>
         </is>
@@ -2716,7 +2724,7 @@
           <t>Questionario padrao respondido (vale p/ os tres).</t>
         </is>
       </c>
-      <c r="F50" s="22" t="inlineStr">
+      <c r="F50" s="23" t="inlineStr">
         <is>
           <t>Documento (escrever 1x)</t>
         </is>
@@ -2756,7 +2764,7 @@
           <t>Rodar a bateria e gerar a gravacao, como fizemos no Print.</t>
         </is>
       </c>
-      <c r="F51" s="18" t="inlineStr">
+      <c r="F51" s="20" t="inlineStr">
         <is>
           <t>Copiar do Print</t>
         </is>
@@ -2796,7 +2804,7 @@
           <t>Publicar a politica de vulnerabilidade (vale p/ os tres).</t>
         </is>
       </c>
-      <c r="F52" s="22" t="inlineStr">
+      <c r="F52" s="23" t="inlineStr">
         <is>
           <t>Documento (escrever 1x)</t>
         </is>
@@ -2836,7 +2844,7 @@
           <t>Cron semanal nos workflows para reavaliar.</t>
         </is>
       </c>
-      <c r="F53" s="21" t="inlineStr">
+      <c r="F53" s="22" t="inlineStr">
         <is>
           <t>Ligar no CI / infra</t>
         </is>
@@ -2892,7 +2900,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>0 de 49 controles feitos. 49 em planejamento. Modelo pronto e testado: Print.</t>
+          <t>0 de 49 controles feitos. Modelo pronto e testado: Print. Parte do zero, do mesmo jeito.</t>
         </is>
       </c>
     </row>
@@ -2962,7 +2970,7 @@
           <t>Toda tabela do servico precisa de tenant_id, e todo SELECT/UPDATE filtrar por ele.</t>
         </is>
       </c>
-      <c r="F5" s="20" t="inlineStr">
+      <c r="F5" s="18" t="inlineStr">
         <is>
           <t>Adaptar do Print</t>
         </is>
@@ -3002,7 +3010,7 @@
           <t>Reusar o login scrypt e a sessao HttpOnly do contas.js.</t>
         </is>
       </c>
-      <c r="F6" s="18" t="inlineStr">
+      <c r="F6" s="20" t="inlineStr">
         <is>
           <t>Copiar do Print</t>
         </is>
@@ -3042,7 +3050,7 @@
           <t>Reusar papeis e a funcao acessoA do banco.js.</t>
         </is>
       </c>
-      <c r="F7" s="18" t="inlineStr">
+      <c r="F7" s="20" t="inlineStr">
         <is>
           <t>Copiar do Print</t>
         </is>
@@ -3082,7 +3090,7 @@
           <t>Guardar arquivo fora da web e servir so por link assinado, como no Print.</t>
         </is>
       </c>
-      <c r="F8" s="20" t="inlineStr">
+      <c r="F8" s="18" t="inlineStr">
         <is>
           <t>Adaptar do Print</t>
         </is>
@@ -3122,7 +3130,7 @@
           <t>Ja vem da borda Railway; garantir HSTS no servidor do servico.</t>
         </is>
       </c>
-      <c r="F9" s="18" t="inlineStr">
+      <c r="F9" s="20" t="inlineStr">
         <is>
           <t>Copiar do Print</t>
         </is>
@@ -3162,7 +3170,7 @@
           <t>Plugar cifra.js na gravacao de conteudo do servico.</t>
         </is>
       </c>
-      <c r="F10" s="18" t="inlineStr">
+      <c r="F10" s="20" t="inlineStr">
         <is>
           <t>Copiar do Print</t>
         </is>
@@ -3202,7 +3210,7 @@
           <t>Dar prazo de validade ao objeto do servico.</t>
         </is>
       </c>
-      <c r="F11" s="20" t="inlineStr">
+      <c r="F11" s="18" t="inlineStr">
         <is>
           <t>Adaptar do Print</t>
         </is>
@@ -3242,7 +3250,7 @@
           <t>Reusar a poda por prazo no caminho de leitura.</t>
         </is>
       </c>
-      <c r="F12" s="18" t="inlineStr">
+      <c r="F12" s="20" t="inlineStr">
         <is>
           <t>Copiar do Print</t>
         </is>
@@ -3282,7 +3290,7 @@
           <t>Excluir tem que apagar metadado e objeto juntos.</t>
         </is>
       </c>
-      <c r="F13" s="20" t="inlineStr">
+      <c r="F13" s="18" t="inlineStr">
         <is>
           <t>Adaptar do Print</t>
         </is>
@@ -3322,7 +3330,7 @@
           <t>Segredos so em variavel de ambiente; nunca no repo.</t>
         </is>
       </c>
-      <c r="F14" s="18" t="inlineStr">
+      <c r="F14" s="20" t="inlineStr">
         <is>
           <t>Copiar do Print</t>
         </is>
@@ -3362,7 +3370,7 @@
           <t>Criar tabela de auditoria e registrar acoes criticas.</t>
         </is>
       </c>
-      <c r="F15" s="18" t="inlineStr">
+      <c r="F15" s="20" t="inlineStr">
         <is>
           <t>Copiar do Print</t>
         </is>
@@ -3402,7 +3410,7 @@
           <t>Reusar papeis: admin, gestor, consultor, leitor.</t>
         </is>
       </c>
-      <c r="F16" s="18" t="inlineStr">
+      <c r="F16" s="20" t="inlineStr">
         <is>
           <t>Copiar do Print</t>
         </is>
@@ -3442,7 +3450,7 @@
           <t>Registrar acesso, criacao, download e exclusao por cliente.</t>
         </is>
       </c>
-      <c r="F17" s="18" t="inlineStr">
+      <c r="F17" s="20" t="inlineStr">
         <is>
           <t>Copiar do Print</t>
         </is>
@@ -3482,7 +3490,7 @@
           <t>Reusar o freio (429) por conta e por origem.</t>
         </is>
       </c>
-      <c r="F18" s="18" t="inlineStr">
+      <c r="F18" s="20" t="inlineStr">
         <is>
           <t>Copiar do Print</t>
         </is>
@@ -3522,7 +3530,7 @@
           <t>Reusar a validacao e o parse de corpo do api.js.</t>
         </is>
       </c>
-      <c r="F19" s="18" t="inlineStr">
+      <c r="F19" s="20" t="inlineStr">
         <is>
           <t>Copiar do Print</t>
         </is>
@@ -3562,7 +3570,7 @@
           <t>Reusar o limite de tamanho de corpo e upload.</t>
         </is>
       </c>
-      <c r="F20" s="18" t="inlineStr">
+      <c r="F20" s="20" t="inlineStr">
         <is>
           <t>Copiar do Print</t>
         </is>
@@ -3602,7 +3610,7 @@
           <t>Aceitar so os tipos de arquivo da lista.</t>
         </is>
       </c>
-      <c r="F21" s="18" t="inlineStr">
+      <c r="F21" s="20" t="inlineStr">
         <is>
           <t>Copiar do Print</t>
         </is>
@@ -3642,7 +3650,7 @@
           <t>Fechar CORS para as origens conhecidas.</t>
         </is>
       </c>
-      <c r="F22" s="18" t="inlineStr">
+      <c r="F22" s="20" t="inlineStr">
         <is>
           <t>Copiar do Print</t>
         </is>
@@ -3682,7 +3690,7 @@
           <t>Copiar os cabecalhos de seguranca do servidor.js.</t>
         </is>
       </c>
-      <c r="F23" s="18" t="inlineStr">
+      <c r="F23" s="20" t="inlineStr">
         <is>
           <t>Copiar do Print</t>
         </is>
@@ -3722,7 +3730,7 @@
           <t>Erro nunca devolve stack; 500 controlado.</t>
         </is>
       </c>
-      <c r="F24" s="18" t="inlineStr">
+      <c r="F24" s="20" t="inlineStr">
         <is>
           <t>Copiar do Print</t>
         </is>
@@ -3762,7 +3770,7 @@
           <t>Reusar o backup do admin.js.</t>
         </is>
       </c>
-      <c r="F25" s="18" t="inlineStr">
+      <c r="F25" s="20" t="inlineStr">
         <is>
           <t>Copiar do Print</t>
         </is>
@@ -3802,7 +3810,7 @@
           <t>Reusar teste-backup.js: destruir e restaurar de verdade.</t>
         </is>
       </c>
-      <c r="F26" s="18" t="inlineStr">
+      <c r="F26" s="20" t="inlineStr">
         <is>
           <t>Copiar do Print</t>
         </is>
@@ -3842,7 +3850,7 @@
           <t>Chaves e banco separados por ambiente (dev/homolog/prod).</t>
         </is>
       </c>
-      <c r="F27" s="21" t="inlineStr">
+      <c r="F27" s="22" t="inlineStr">
         <is>
           <t>Ligar no CI / infra</t>
         </is>
@@ -3882,7 +3890,7 @@
           <t>Rodar os mesmos testes no CI antes de subir.</t>
         </is>
       </c>
-      <c r="F28" s="21" t="inlineStr">
+      <c r="F28" s="22" t="inlineStr">
         <is>
           <t>Ligar no CI / infra</t>
         </is>
@@ -3922,7 +3930,7 @@
           <t>Exigir revisao de PR antes do main.</t>
         </is>
       </c>
-      <c r="F29" s="21" t="inlineStr">
+      <c r="F29" s="22" t="inlineStr">
         <is>
           <t>Ligar no CI / infra</t>
         </is>
@@ -3962,7 +3970,7 @@
           <t>Ligar o codeql.yml no repositorio do servico.</t>
         </is>
       </c>
-      <c r="F30" s="21" t="inlineStr">
+      <c r="F30" s="22" t="inlineStr">
         <is>
           <t>Ligar no CI / infra</t>
         </is>
@@ -4002,7 +4010,7 @@
           <t>Rodar npm audit (ou equivalente) no CI.</t>
         </is>
       </c>
-      <c r="F31" s="21" t="inlineStr">
+      <c r="F31" s="22" t="inlineStr">
         <is>
           <t>Ligar no CI / infra</t>
         </is>
@@ -4042,7 +4050,7 @@
           <t>Ligar o secret scanning do GitHub e revisar o .gitignore.</t>
         </is>
       </c>
-      <c r="F32" s="21" t="inlineStr">
+      <c r="F32" s="22" t="inlineStr">
         <is>
           <t>Ligar no CI / infra</t>
         </is>
@@ -4082,7 +4090,7 @@
           <t>Fixar versoes e ligar o Dependabot.</t>
         </is>
       </c>
-      <c r="F33" s="21" t="inlineStr">
+      <c r="F33" s="22" t="inlineStr">
         <is>
           <t>Ligar no CI / infra</t>
         </is>
@@ -4122,7 +4130,7 @@
           <t>Deixar a identidade pronta para SSO (sso.js ja prepara).</t>
         </is>
       </c>
-      <c r="F34" s="18" t="inlineStr">
+      <c r="F34" s="20" t="inlineStr">
         <is>
           <t>Copiar do Print</t>
         </is>
@@ -4162,7 +4170,7 @@
           <t>Escrever o processo de resposta a incidente (vale p/ os tres).</t>
         </is>
       </c>
-      <c r="F35" s="22" t="inlineStr">
+      <c r="F35" s="23" t="inlineStr">
         <is>
           <t>Documento (escrever 1x)</t>
         </is>
@@ -4202,7 +4210,7 @@
           <t>Formalizar o tratamento LGPD e reusar o mascaramento de dado sensivel.</t>
         </is>
       </c>
-      <c r="F36" s="22" t="inlineStr">
+      <c r="F36" s="23" t="inlineStr">
         <is>
           <t>Documento (escrever 1x)</t>
         </is>
@@ -4242,7 +4250,7 @@
           <t>Listar quais dados o servico trata (curto, por servico).</t>
         </is>
       </c>
-      <c r="F37" s="22" t="inlineStr">
+      <c r="F37" s="23" t="inlineStr">
         <is>
           <t>Documento (escrever 1x)</t>
         </is>
@@ -4282,7 +4290,7 @@
           <t>Listar terceiros que processam dados (Railway etc, vale p/ os tres).</t>
         </is>
       </c>
-      <c r="F38" s="22" t="inlineStr">
+      <c r="F38" s="23" t="inlineStr">
         <is>
           <t>Documento (escrever 1x)</t>
         </is>
@@ -4322,7 +4330,7 @@
           <t>Copiar sso.js e teste-sso.js e apontar para o provedor do cliente.</t>
         </is>
       </c>
-      <c r="F39" s="18" t="inlineStr">
+      <c r="F39" s="20" t="inlineStr">
         <is>
           <t>Copiar do Print</t>
         </is>
@@ -4362,7 +4370,7 @@
           <t>Adaptar o dast.js as rotas do servico e rodar no CI.</t>
         </is>
       </c>
-      <c r="F40" s="21" t="inlineStr">
+      <c r="F40" s="22" t="inlineStr">
         <is>
           <t>Ligar no CI / infra</t>
         </is>
@@ -4402,7 +4410,7 @@
           <t>Agendar pentest externo (fora do time).</t>
         </is>
       </c>
-      <c r="F41" s="23" t="inlineStr">
+      <c r="F41" s="24" t="inlineStr">
         <is>
           <t>Arquitetura / externo</t>
         </is>
@@ -4442,7 +4450,7 @@
           <t>Se o servico usa modelo, reusar injecao.js; senao, nao se aplica.</t>
         </is>
       </c>
-      <c r="F42" s="18" t="inlineStr">
+      <c r="F42" s="20" t="inlineStr">
         <is>
           <t>Copiar do Print</t>
         </is>
@@ -4482,7 +4490,7 @@
           <t>Reusar injecao.js: conteudo externo entra como dado, nunca ordem.</t>
         </is>
       </c>
-      <c r="F43" s="18" t="inlineStr">
+      <c r="F43" s="20" t="inlineStr">
         <is>
           <t>Copiar do Print</t>
         </is>
@@ -4522,7 +4530,7 @@
           <t>O modelo nao executa acao; so descreve.</t>
         </is>
       </c>
-      <c r="F44" s="23" t="inlineStr">
+      <c r="F44" s="24" t="inlineStr">
         <is>
           <t>Arquitetura / externo</t>
         </is>
@@ -4562,7 +4570,7 @@
           <t>Reusar a conferencia de saida do injecao.js.</t>
         </is>
       </c>
-      <c r="F45" s="18" t="inlineStr">
+      <c r="F45" s="20" t="inlineStr">
         <is>
           <t>Copiar do Print</t>
         </is>
@@ -4602,7 +4610,7 @@
           <t>Documentar a arquitetura e os controles do servico.</t>
         </is>
       </c>
-      <c r="F46" s="22" t="inlineStr">
+      <c r="F46" s="23" t="inlineStr">
         <is>
           <t>Documento (escrever 1x)</t>
         </is>
@@ -4642,7 +4650,7 @@
           <t>Desenhar o fluxo de dados do servico.</t>
         </is>
       </c>
-      <c r="F47" s="22" t="inlineStr">
+      <c r="F47" s="23" t="inlineStr">
         <is>
           <t>Documento (escrever 1x)</t>
         </is>
@@ -4682,7 +4690,7 @@
           <t>Marcar as fronteiras de confianca do servico.</t>
         </is>
       </c>
-      <c r="F48" s="22" t="inlineStr">
+      <c r="F48" s="23" t="inlineStr">
         <is>
           <t>Documento (escrever 1x)</t>
         </is>
@@ -4722,7 +4730,7 @@
           <t>FAQ de seguranca padrao (vale p/ os tres).</t>
         </is>
       </c>
-      <c r="F49" s="22" t="inlineStr">
+      <c r="F49" s="23" t="inlineStr">
         <is>
           <t>Documento (escrever 1x)</t>
         </is>
@@ -4762,7 +4770,7 @@
           <t>Questionario padrao respondido (vale p/ os tres).</t>
         </is>
       </c>
-      <c r="F50" s="22" t="inlineStr">
+      <c r="F50" s="23" t="inlineStr">
         <is>
           <t>Documento (escrever 1x)</t>
         </is>
@@ -4802,7 +4810,7 @@
           <t>Rodar a bateria e gerar a gravacao, como fizemos no Print.</t>
         </is>
       </c>
-      <c r="F51" s="18" t="inlineStr">
+      <c r="F51" s="20" t="inlineStr">
         <is>
           <t>Copiar do Print</t>
         </is>
@@ -4842,7 +4850,7 @@
           <t>Publicar a politica de vulnerabilidade (vale p/ os tres).</t>
         </is>
       </c>
-      <c r="F52" s="22" t="inlineStr">
+      <c r="F52" s="23" t="inlineStr">
         <is>
           <t>Documento (escrever 1x)</t>
         </is>
@@ -4882,7 +4890,7 @@
           <t>Cron semanal nos workflows para reavaliar.</t>
         </is>
       </c>
-      <c r="F53" s="21" t="inlineStr">
+      <c r="F53" s="22" t="inlineStr">
         <is>
           <t>Ligar no CI / infra</t>
         </is>

</xml_diff>